<commit_message>
Workbook: complete actual hours, add hour basis, CDU Horizon test
All actual-hour cells are filled. Column I of Billable tasks says whether
each figure was entered by the member, taken from the time log, or is a
retrospective estimate. Totals add shared-task hours without counting
Ashesh's share twice (Ashesh 80, Susan 9.5, Milan 41.0, group 130.5).
RTM records the CDU Horizon virtual desktop test; the designated VM test
is still pending.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HIT339_G16_Traceability_and_Hours.xlsx
+++ b/docs/HIT339_G16_Traceability_and_Hours.xlsx
@@ -554,7 +554,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -572,7 +571,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Billable tasks: tasks, allocations, 12 October planning estimates and the actual hours each member entered. Ashesh's actual hours are retrospective estimates made on 16 October 2026 from the commits and pull requests, not recorded timesheets. Estimates are not hours worked.</t>
+          <t>Billable tasks: tasks, allocations, 12 October planning estimates and actual hours. Column I gives the basis of each actual figure: entered by the member, from the time log, or a retrospective estimate (made on 16 October 2026). Estimates are not recorded times.</t>
         </is>
       </c>
     </row>
@@ -590,11 +589,10 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yellow cells are hours still to be entered by the member concerned.</t>
+          <t>All actual-hour cells are now filled. The group portfolio (Part 9) shows the same figures.</t>
         </is>
       </c>
     </row>
@@ -698,22 +696,22 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>374 tests passed on macOS and on Milan's and Susan's Windows 11 PCs (16 Oct)</t>
+          <t>374 tests passed on macOS, on Milan's and Susan's Windows 11 PCs and on a CDU Horizon Windows virtual desktop (16 Oct)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Installation Manual step 9: Windows PC test record and screenshots</t>
+          <t>Installation Manual step 9: Windows PC test record and CDU Horizon screenshots</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Met on Windows PCs; designated VM test pending</t>
+          <t>Met on Windows PCs and a CDU Horizon virtual desktop; designated VM test pending</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Designated VM test being arranged by Susan; results pending</t>
+          <t>Not confirmed whether the CDU Horizon desktop is the designated VM; Susan arranging the designated VM test</t>
         </is>
       </c>
     </row>
@@ -959,7 +957,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Ashesh's actual hours are retrospective estimates; some of Susan's and Milan's portfolio tasks have no hours entered</t>
+          <t>Actual hours not from the time log are retrospective estimates (column I of Billable tasks)</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1458,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Full suite on .NET 10: macOS and two Windows 11 PCs</t>
+          <t>Full suite on .NET 10: macOS, two Windows 11 PCs and a CDU Horizon virtual desktop</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1507,7 +1505,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Windows 11 PC tests (Milan, Susan): 374 passed; nine installation checks passed</t>
+          <t>Windows 11 PCs (Milan, Susan): 374 passed, nine installation checks passed; CDU Horizon virtual desktop (Ashesh): 374 passed, site ran, PDF report opened</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1522,7 +1520,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Susan is arranging the designated VM test</t>
+          <t>Not confirmed whether the CDU Horizon desktop is the designated VM; Susan arranging the designated VM test</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2366,6 +2364,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2409,6 +2408,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Actual hours basis</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2434,7 +2438,9 @@
       <c r="E2" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F2" s="4" t="n"/>
+      <c r="F2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Agreed scope and section owners</t>
@@ -2443,6 +2449,11 @@
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Done before 11 Oct</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate: Susan 1.5, Milan 1.5</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2481,9 @@
       <c r="E3" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="4" t="n"/>
+      <c r="F3" s="3" t="n">
+        <v>2.5</v>
+      </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Coordination records</t>
@@ -2479,6 +2492,11 @@
       <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Done; see coordination records</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate: Susan 1, Milan 1.5</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2524,9 @@
       <c r="E4" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F4" s="4" t="n"/>
+      <c r="F4" s="3" t="n">
+        <v>1.5</v>
+      </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Test records</t>
@@ -2514,7 +2534,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Done: macOS (Ashesh), Windows 11 PCs (Milan, Susan); designated VM test pending</t>
+          <t>Done: macOS (Ashesh), Windows 11 PCs (Milan, Susan), CDU Horizon virtual desktop (Ashesh); designated VM test pending</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Milan, time log</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2567,9 @@
       <c r="E5" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F5" s="4" t="n"/>
+      <c r="F5" s="3" t="n">
+        <v>1.25</v>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Submitted portfolio and repository</t>
@@ -2551,6 +2578,11 @@
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Ready for final review</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Susan 0.25, time log; Milan 1, est.</t>
         </is>
       </c>
     </row>
@@ -2591,6 +2623,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2629,6 +2666,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2667,6 +2709,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2705,6 +2752,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2743,6 +2795,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2781,6 +2838,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2819,6 +2881,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2857,6 +2924,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2895,6 +2967,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2933,6 +3010,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2971,6 +3053,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3009,6 +3096,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3047,6 +3139,11 @@
           <t>Done, merged (PR #2)</t>
         </is>
       </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -3085,6 +3182,11 @@
           <t>Done, merged (PR #1)</t>
         </is>
       </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3123,6 +3225,11 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -3163,6 +3270,7 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -3203,6 +3311,7 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -3243,6 +3352,7 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -3283,6 +3393,7 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -3323,6 +3434,7 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3363,6 +3475,7 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -3388,10 +3501,8 @@
       <c r="E27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>0 (not needed)</t>
-        </is>
+      <c r="F27" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
@@ -3401,6 +3512,11 @@
       <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Not needed: Section 2 added no migration</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Not needed</t>
         </is>
       </c>
     </row>
@@ -3441,6 +3557,11 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3479,6 +3600,11 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3517,6 +3643,11 @@
           <t>Done, merged (PR #4)</t>
         </is>
       </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3555,6 +3686,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3593,6 +3729,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -3631,6 +3772,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3669,6 +3815,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -3707,6 +3858,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -3745,6 +3901,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -3783,6 +3944,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -3821,6 +3987,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -3859,6 +4030,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -3897,6 +4073,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -3935,6 +4116,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -3973,6 +4159,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -4011,6 +4202,11 @@
           <t>Done, merged (PR #3)</t>
         </is>
       </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -4049,6 +4245,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -4087,6 +4288,11 @@
           <t>Done, merged (PR #7)</t>
         </is>
       </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -4125,6 +4331,11 @@
           <t>Done 12 Oct, before PR #2 was merged</t>
         </is>
       </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -4165,6 +4376,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -4205,6 +4421,11 @@
           <t>Done 15 Oct; reported to Ashesh</t>
         </is>
       </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -4245,6 +4466,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -4285,6 +4511,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -4325,6 +4556,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -4365,6 +4601,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -4405,6 +4646,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -4445,6 +4691,11 @@
           <t>Done, merged (PR #6)</t>
         </is>
       </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -4483,6 +4734,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -4521,6 +4777,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -4559,6 +4820,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -4597,6 +4863,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -4635,6 +4906,11 @@
           <t>Done, merged (PR #5)</t>
         </is>
       </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -4660,7 +4936,9 @@
       <c r="E60" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F60" s="4" t="n"/>
+      <c r="F60" s="3" t="n">
+        <v>1.5</v>
+      </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Patron User Guide</t>
@@ -4669,6 +4947,11 @@
       <c r="H60" s="3" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4979,9 @@
       <c r="E61" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F61" s="4" t="n"/>
+      <c r="F61" s="3" t="n">
+        <v>1.5</v>
+      </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
           <t>Requirements</t>
@@ -4705,6 +4990,11 @@
       <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate</t>
         </is>
       </c>
     </row>
@@ -4745,6 +5035,11 @@
           <t>Windows 11 PC tests done (Milan, Susan; see step 9); designated VM test pending, being arranged by Susan</t>
         </is>
       </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>Entered by the member</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -4770,7 +5065,9 @@
       <c r="E63" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F63" s="4" t="n"/>
+      <c r="F63" s="3" t="n">
+        <v>0.25</v>
+      </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Team Contract</t>
@@ -4779,6 +5076,11 @@
       <c r="H63" s="3" t="inlineStr">
         <is>
           <t>Done; signed by Susan and Milan, Ashesh's signature to be added</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate</t>
         </is>
       </c>
     </row>
@@ -4806,7 +5108,9 @@
       <c r="E64" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F64" s="4" t="n"/>
+      <c r="F64" s="3" t="n">
+        <v>1.5</v>
+      </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Coordination records</t>
@@ -4815,6 +5119,11 @@
       <c r="H64" s="3" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate</t>
         </is>
       </c>
     </row>
@@ -4842,7 +5151,9 @@
       <c r="E65" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F65" s="4" t="n"/>
+      <c r="F65" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Strengths and weaknesses</t>
@@ -4851,6 +5162,11 @@
       <c r="H65" s="3" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate</t>
         </is>
       </c>
     </row>
@@ -4891,6 +5207,11 @@
           <t>Done; repository made public on 16 Oct, so no invitation is needed</t>
         </is>
       </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4929,6 +5250,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -4969,6 +5295,11 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -5007,6 +5338,11 @@
       <c r="H69" s="3" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective estimate (Ashesh)</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5032,6 +5368,8 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5060,6 +5398,16 @@
           <t>Actual hours (own tasks)</t>
         </is>
       </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Actual hours (shared tasks)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Actual total</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5083,6 +5431,13 @@
         <f>SUMIFS('Billable tasks'!F:F,'Billable tasks'!D:D,"Ashesh*")</f>
         <v/>
       </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <f>E2+F2</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5106,6 +5461,13 @@
         <f>SUMIFS('Billable tasks'!F:F,'Billable tasks'!D:D,"Susan*")</f>
         <v/>
       </c>
+      <c r="F3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="G3">
+        <f>E3+F3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5129,6 +5491,13 @@
         <f>SUMIFS('Billable tasks'!F:F,'Billable tasks'!D:D,"Milan*")</f>
         <v/>
       </c>
+      <c r="F4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G4">
+        <f>E4+F4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5170,6 +5539,14 @@
         <f>SUM(E2:E4)</f>
         <v/>
       </c>
+      <c r="F6" s="6">
+        <f>SUM(F2:F4)</f>
+        <v/>
+      </c>
+      <c r="G6" s="6">
+        <f>SUM(G2:G4)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5181,7 +5558,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Susan's total of 3.75 hours in the portfolio also includes 0.25 hours on the shared task G-04 (see Time log). Ashesh's 80 hours are retrospective estimates.</t>
+          <t>Shared tasks (G-01 to G-04) list only Susan's and Milan's hours; Ashesh's part is already counted in his own tasks, so nothing is counted twice. Expected actual totals: Ashesh 80, Susan 9.5, Milan 41.0, group 130.5. Ashesh's hours and figures marked as estimates in Billable tasks are retrospective estimates, not recorded times.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: record the virtual machine test on CDU's Horizon IT Desktop
The VM test was done by Ashesh on CDU's Horizon IT Desktop, a
university-hosted Windows virtual desktop, on 16 Oct 2026 at b695674
(374 tests passed, site ran, Fine Revenue Audit PDF opened).
README and workbook no longer describe the VM test as pending.
Documentation only; no application changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HIT339_G16_Traceability_and_Hours.xlsx
+++ b/docs/HIT339_G16_Traceability_and_Hours.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Version 1.1, 16 October 2026. Release documented: main at b695674 (application code as at 55fbc1d). Synchronised with the group portfolio.</t>
+          <t>Version 1.2, 16 October 2026. Application release documented: b695674 (application code as at 55fbc1d). Synchronised with the group portfolio.</t>
         </is>
       </c>
     </row>
@@ -696,22 +696,22 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>374 tests passed on macOS, on Milan's and Susan's Windows 11 PCs and on a CDU Horizon Windows virtual desktop (16 Oct)</t>
+          <t>374 tests passed on macOS, on Milan's and Susan's Windows 11 PCs and on CDU's Horizon IT Desktop, a university-hosted Windows virtual desktop (16 Oct, commit b695674)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Installation Manual step 9: Windows PC test record and CDU Horizon screenshots</t>
+          <t>Installation Manual step 9: Windows PC test record and virtual machine screenshots</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Met on Windows PCs and a CDU Horizon virtual desktop; designated VM test pending</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Not confirmed whether the CDU Horizon desktop is the designated VM; Susan arranging the designated VM test</t>
+          <t>On the virtual machine: clone, build, tests, site running and a PDF report; the full nine checks were done on the two Windows PCs</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Full suite on .NET 10: macOS, two Windows 11 PCs and a CDU Horizon virtual desktop</t>
+          <t>Full suite on .NET 10: macOS, two Windows 11 PCs and CDU's Horizon IT Desktop</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1471,11 +1471,7 @@
           <t>Met</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Designated VM test pending</t>
-        </is>
-      </c>
+      <c r="I20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1505,7 +1501,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Windows 11 PCs (Milan, Susan): 374 passed, nine installation checks passed; CDU Horizon virtual desktop (Ashesh): 374 passed, site ran, PDF report opened</t>
+          <t>Windows 11 PCs (Milan, Susan): 374 passed, nine installation checks passed; CDU's Horizon IT Desktop, a university-hosted Windows virtual desktop (Ashesh, b695674): 374 passed, site ran, PDF report opened</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1515,14 +1511,10 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Partly met: designated VM test pending</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Not confirmed whether the CDU Horizon desktop is the designated VM; Susan arranging the designated VM test</t>
-        </is>
-      </c>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2534,7 +2526,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Done: macOS (Ashesh), Windows 11 PCs (Milan, Susan), CDU Horizon virtual desktop (Ashesh); designated VM test pending</t>
+          <t>Done: macOS (Ashesh), Windows 11 PCs (Milan, Susan), CDU's Horizon IT Desktop (Ashesh)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -5011,7 +5003,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Deployment and test on the designated VM</t>
+          <t>Deployment and test on the virtual machine</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -5032,7 +5024,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>Windows 11 PC tests done (Milan, Susan; see step 9); designated VM test pending, being arranged by Susan</t>
+          <t>Windows 11 PC tests done (Milan, Susan; see step 9); virtual machine test done by Ashesh on CDU's Horizon IT Desktop (16 Oct)</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">

</xml_diff>